<commit_message>
Set the Patriot limit to 8 batteries at 2 sites each in the economic-research workbook and spec
PATRIOT_MAX is now 8, so Patriot can cover all 16 sites. The hand checks cover the 8-battery case (all sites covered, none uncovered), and spec.md and the README match. Reference results are unchanged because the optimum never needs more than 2 batteries at the workbook's placeholder battery cost.

Verified in Excel against the Python optimizer on all 10 reference cases; Solver was not run.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/capabilities/economic-research/model.xlsx
+++ b/capabilities/economic-research/model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\richi\AppData\Local\Temp\mx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{42BD17A9-959F-47D2-8804-EA03A9B39F73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{402FC98C-65C2-4285-BDD0-4C8BB6AD069A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -283,7 +283,7 @@
     <t>Built from capabilities/economic-research/spec.md. Blue = input (all DRAFT placeholders until sourced). Yellow = decision cell (Solver changes these). Black = formula. Money in USD millions ($M).</t>
   </si>
   <si>
-    <t>HOW TO USE: replace blue inputs with sourced figures, pick ACTIVE_RAID and BUDGET, then Data &gt; Solver &gt; Solve (the Solver setup is saved in this sheet). Site constraints (16 sites, Patriot at 2 sites per battery, at most 4 batteries) are in rows 98-141 and the QC grid; QU (rows 35-38) is the grid at sites without Patriot cover.</t>
+    <t>HOW TO USE: replace blue inputs with sourced figures, pick ACTIVE_RAID and BUDGET, then Data &gt; Solver &gt; Solve (the Solver setup is saved in this sheet). Site constraints (16 sites, Patriot at 2 sites per battery, at most 8 batteries) are in rows 98-141 and the QC grid; QU (rows 35-38) is the grid at sites without Patriot cover.</t>
   </si>
   <si>
     <t>INPUTS - per interceptor (DRAFT: secondary-source ranges and placeholder assumptions)</t>
@@ -829,7 +829,7 @@
     <t>batteries</t>
   </si>
   <si>
-    <t>User-specified: the limit on Patriot batteries on Guam.</t>
+    <t>User-specified: 8 Patriot batteries on Guam (the limit; the model may build fewer). At 2 sites each, 8 batteries cover all 16 sites.</t>
   </si>
   <si>
     <t>AEGIS_SITES</t>
@@ -967,16 +967,16 @@
     <t>HAND CHECK - site constraints (build audit): formula vs. hand math</t>
   </si>
   <si>
-    <t>4 batteries x 2 sites = 8 covered sites, half of 16 (COVERED_FRACTION = 0.5)</t>
-  </si>
-  <si>
-    <t>40 ballistic threats, half arriving at covered sites: R_COVERED = 20</t>
-  </si>
-  <si>
-    <t>4 Patriot batteries x 6 launchers x 16 CRI = 384 PAC-3 CRI at most</t>
-  </si>
-  <si>
-    <t>Uncovered share: 8 of 16 sites uncovered, so (1 - 0.5) x 50 drones = 25</t>
+    <t>8 batteries x 2 sites = 16 covered sites = every site (COVERED_FRACTION = 1)</t>
+  </si>
+  <si>
+    <t>40 ballistic threats, all arriving at covered sites: R_COVERED = 40 (R_UNCOVERED = 0)</t>
+  </si>
+  <si>
+    <t>8 Patriot batteries x 6 launchers x 16 CRI = 768 PAC-3 CRI at most</t>
+  </si>
+  <si>
+    <t>With 4 batteries, 8 of 16 sites are uncovered, so (1 - 0.5) x 50 drones = 25 uncovered</t>
   </si>
   <si>
     <t>Raid scenarios and results log</t>
@@ -1033,7 +1033,7 @@
     <t>A ballistic-heavy (USE_MIN 0.98)</t>
   </si>
   <si>
-    <t>Source: scipy.optimize.milp run by Claude on 2026-10-08 with the Model sheet inputs as built, with the site constraints (16 sites, raids spread evenly, 2 sites per Patriot battery, at most 4 batteries, Patriot interceptors only at covered sites); tangent-line approximation of D, protection re-evaluated exactly. These replace the earlier results that had no site limits. Illustrative only.</t>
+    <t>Source: scipy.optimize.milp run by Claude on 2026-10-08 with the Model sheet inputs as built, with the site constraints (16 sites, raids spread evenly, 2 sites per Patriot battery, at most 8 batteries, Patriot interceptors only at covered sites); tangent-line approximation of D, protection re-evaluated exactly. These replace the earlier results that had no site limits. Illustrative only.</t>
   </si>
   <si>
     <t>MY SOLVER RUNS - record each Excel Solver result here</t>
@@ -1153,7 +1153,7 @@
     <t>Constraint 11</t>
   </si>
   <si>
-    <t>PATRIOT_BATTERIES (C41) &lt;= PATRIOT_MAX (B102) - the Guam limit of 4 batteries; 2 sites each, so at most 8 of 16 sites have Patriot cover</t>
+    <t>PATRIOT_BATTERIES (C41) &lt;= PATRIOT_MAX (B102) - the limit of 8 batteries; 2 sites each, so 8 batteries cover all 16 sites</t>
   </si>
   <si>
     <t>Constraint 12</t>
@@ -3768,7 +3768,7 @@
         <v>182</v>
       </c>
       <c r="B102" s="30">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" s="2"/>
@@ -4466,11 +4466,11 @@
         <v>230</v>
       </c>
       <c r="B138" s="27">
-        <f>MIN(16,2*4)/16</f>
-        <v>0.5</v>
+        <f>MIN(16,2*8)/16</f>
+        <v>1</v>
       </c>
       <c r="C138" s="10">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D138" s="2" t="b">
         <f>B138=C138</f>
@@ -4487,11 +4487,11 @@
         <v>231</v>
       </c>
       <c r="B139" s="27">
-        <f>40*(MIN(16,2*4)/16)</f>
-        <v>20</v>
+        <f>40*(MIN(16,2*8)/16)</f>
+        <v>40</v>
       </c>
       <c r="C139" s="10">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="D139" s="2" t="b">
         <f>B139=C139</f>
@@ -4508,11 +4508,11 @@
         <v>232</v>
       </c>
       <c r="B140" s="27">
-        <f>4*6*16</f>
-        <v>384</v>
+        <f>8*6*16</f>
+        <v>768</v>
       </c>
       <c r="C140" s="10">
-        <v>384</v>
+        <v>768</v>
       </c>
       <c r="D140" s="2" t="b">
         <f>B140=C140</f>

</xml_diff>

<commit_message>
Finish the repo: final draft, README row, workbook with exact reference results, Solver runs
Replaces the 2026-10-10 draft with revised_5, adds the cost-exchange-ratio engagement to the root README, and updates the workbook, reference optimizer, spec and analysis note. The reference optimizer now polishes the integer program's solution with an exact local search that breaks ties toward the cheaper loadout: Patriot-only in the cruise-heavy raid is 88.58 percent (89, not 88), the current plan costs 3.1 billion dollars in every raid, and the optimal mix reaches 97.5, 95.0 and 59.3 percent. The workbook's saved Solver options are fixed (Multistart and Require Bounds off) and the Solver runs are recorded; Option 3 did not finish.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/capabilities/economic-research/model.xlsx
+++ b/capabilities/economic-research/model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\richi\AppData\Local\Temp\mx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{18976A0C-88FC-4CDF-883A-7A9AE54E329A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CEECCF18-1DEC-4292-B3C8-F2C57E659AC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -140,13 +140,13 @@
     <definedName name="solver_lhs9" localSheetId="0" hidden="1">Model!$B$67:$G$67</definedName>
     <definedName name="solver_lin" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_mip" localSheetId="0" hidden="1">2147483647</definedName>
-    <definedName name="solver_msl" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_msl" localSheetId="0">2</definedName>
     <definedName name="solver_neg" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_nod" localSheetId="0" hidden="1">2147483647</definedName>
     <definedName name="solver_num" localSheetId="0">20</definedName>
     <definedName name="solver_opt" localSheetId="0" hidden="1">Model!$B$65</definedName>
     <definedName name="solver_pre" localSheetId="0" hidden="1">0.000001</definedName>
-    <definedName name="solver_rbv" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_rbv" localSheetId="0">2</definedName>
     <definedName name="solver_rel1" localSheetId="0" hidden="1">4</definedName>
     <definedName name="solver_rel10" localSheetId="0" hidden="1">3</definedName>
     <definedName name="solver_rel11" localSheetId="0">4</definedName>
@@ -294,7 +294,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="398">
   <si>
     <t>Guam interceptor loadout - economic research model (inputs from Table 1 of the paper, 2026-10-10; site constraints, kill rate and options added)</t>
   </si>
@@ -1121,7 +1121,7 @@
     <t>Table 2 of the paper: where each number comes from</t>
   </si>
   <si>
-    <t>Each Table 2 cell is the PROTECTION cell (Model!B65) after setting OPTION (Model!B154), ACTIVE_RAID (Model!B31) and BUDGET (Model!B23 = 8,000) and solving. The reference values on the Scenarios sheet (rows 13-21) come from an external integer solver (reference-optimizer.py, in this folder); column E checks each of the paper's rounded values against them (FALSE = the paper's number differs from the workbook).</t>
+    <t>Each Table 2 cell is the PROTECTION cell (Model!B65) after setting OPTION (Model!B154), ACTIVE_RAID (Model!B31) and BUDGET (Model!B23 = 8,000) and solving. The reference values on the Scenarios sheet (rows 13-21) come from an external integer solver followed by an exact local search (reference-optimizer.py, in this folder); column E checks each of the paper's rounded values against them (FALSE = the paper's number differs from the workbook).</t>
   </si>
   <si>
     <t>Inputs are Table 1 of the paper; the 50% kill probability, raid sizes, damage weights and the even spread of threats over 16 sites are placeholders. Options 2 and 3 are re-solved for each raid; Option 1 is one fixed purchase.</t>
@@ -1280,6 +1280,75 @@
     <t>Notes</t>
   </si>
   <si>
+    <t>Option 1, A ballistic-heavy</t>
+  </si>
+  <si>
+    <t>Yes (same)</t>
+  </si>
+  <si>
+    <t>Excel Solver (GRG Nonlinear), started from an evenly spread allocation; code 14: Solver found an integer solution within tolerance; all constraints satisfied; 2.5 s; ALL_VALID True. Run by Claude, 2026-10-10.</t>
+  </si>
+  <si>
+    <t>Excel Solver (GRG Nonlinear), started from the reference solution; code 14: Solver found an integer solution within tolerance; all constraints satisfied; 2.2 s; ALL_VALID True. Run by Claude, 2026-10-10.</t>
+  </si>
+  <si>
+    <t>No: 29.1 points below</t>
+  </si>
+  <si>
+    <t>Excel Solver (GRG Nonlinear), started from a rough point (all interceptors in the first class); code 1: Solver converged to the current solution; all constraints satisfied; 1.4 s; ALL_VALID True. Run by Claude, 2026-10-10.</t>
+  </si>
+  <si>
+    <t>Option 1, B cruise-heavy</t>
+  </si>
+  <si>
+    <t>Excel Solver (GRG Nonlinear), started from the reference solution; code 0: Solver found a solution; all constraints and optimality conditions satisfied; 2 s; ALL_VALID True. Run by Claude, 2026-10-10.</t>
+  </si>
+  <si>
+    <t>Option 1, C drone saturation</t>
+  </si>
+  <si>
+    <t>Excel Solver (GRG Nonlinear), started from the reference solution; code 14: Solver found an integer solution within tolerance; all constraints satisfied; 2.1 s; ALL_VALID True. Run by Claude, 2026-10-10.</t>
+  </si>
+  <si>
+    <t>Option 2, A ballistic-heavy</t>
+  </si>
+  <si>
+    <t>Excel Solver (GRG Nonlinear), started from the reference solution; code 0: Solver found a solution; all constraints and optimality conditions satisfied; 1.3 s; ALL_VALID True. Run by Claude, 2026-10-10.</t>
+  </si>
+  <si>
+    <t>Excel Solver (GRG Nonlinear), started from a rough point (all interceptors in the first class); code 0: Solver found a solution; all constraints and optimality conditions satisfied; 2.6 s; ALL_VALID True. Run by Claude, 2026-10-10.</t>
+  </si>
+  <si>
+    <t>Option 2, B cruise-heavy</t>
+  </si>
+  <si>
+    <t>Excel Solver (GRG Nonlinear), started from the reference solution; code 0: Solver found a solution; all constraints and optimality conditions satisfied; 1.6 s; ALL_VALID True. Run by Claude, 2026-10-10.</t>
+  </si>
+  <si>
+    <t>Option 2, C drone saturation</t>
+  </si>
+  <si>
+    <t>Option 3, A ballistic-heavy</t>
+  </si>
+  <si>
+    <t>Did not finish</t>
+  </si>
+  <si>
+    <t>Excel Solver (GRG Nonlinear), started from the reference solution: no result within the 60 s limit plus a 240 s wait; the reference solution is feasible (ALL_VALID TRUE) but Solver could not confirm or improve it. Run by Claude, 2026-10-10.</t>
+  </si>
+  <si>
+    <t>Option 3, B cruise-heavy</t>
+  </si>
+  <si>
+    <t>Option 3, C drone saturation</t>
+  </si>
+  <si>
+    <t>No: 0.1 points below</t>
+  </si>
+  <si>
+    <t>Excel Solver (GRG Nonlinear), started from the reference solution; code 14: Solver found an integer solution within tolerance; all constraints satisfied; 4.4 s; ALL_VALID True. Run by Claude, 2026-10-10.</t>
+  </si>
+  <si>
     <t>Solver setup (saved in the Model sheet; open Data &gt; Solver to see it)</t>
   </si>
   <si>
@@ -1298,7 +1367,7 @@
     <t>Engine</t>
   </si>
   <si>
-    <t>GRG Nonlinear (the objective uses EXP, so Simplex LP cannot be used), with Multistart on. Integer optimality tolerance 0%. Not run in the build (Solver hangs headless).</t>
+    <t>GRG Nonlinear (the objective uses EXP, so Simplex LP cannot be used); Multistart OFF and Require Bounds OFF (with them ON every Solve stops with 'All variables must have both upper and lower bounds'); integer optimality tolerance 0%; Max Time 60 s. Run from the Solver dialog or SolverSolve.</t>
   </si>
   <si>
     <t>Constraint 1</t>
@@ -1382,7 +1451,7 @@
     <t>Known limits</t>
   </si>
   <si>
-    <t>Inputs are placeholders. Kill probabilities and raid sizes are assumptions, not data, and so is the even spread of threats over the 16 sites. GRG on an integer problem can stop at a local optimum - that is why the external reference results exist.</t>
+    <t>Inputs are placeholders. Kill probabilities and raid sizes are assumptions, not data, and so is the even spread of threats over the 16 sites. GRG with integer variables can stall at a poor point from a bad start and cannot finish the Option 3 problem in reasonable time; that is why the external reference results exist. See the Scenarios sheet, MY SOLVER RUNS, for what Solver did on 2026-10-10.</t>
   </si>
   <si>
     <t>Constraint 11</t>
@@ -1425,13 +1494,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.0"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
     <numFmt numFmtId="168" formatCode="0.000"/>
     <numFmt numFmtId="169" formatCode="0.0"/>
+    <numFmt numFmtId="170" formatCode="0.0000%"/>
+    <numFmt numFmtId="171" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="14" x14ac:knownFonts="1">
     <font>
@@ -1576,7 +1647,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1623,6 +1694,8 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="169" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2866,11 +2939,11 @@
       </c>
       <c r="B45" s="21">
         <f t="shared" ref="B45:G45" si="0">SUM(B35:B38)+SUM(B108:B111)</f>
-        <v>322</v>
+        <v>613</v>
       </c>
       <c r="C45" s="21">
         <f t="shared" si="0"/>
-        <v>257</v>
+        <v>0</v>
       </c>
       <c r="D45" s="21">
         <f t="shared" si="0"/>
@@ -2902,11 +2975,11 @@
       </c>
       <c r="B46" s="22">
         <f t="shared" ref="B46:G46" si="1">B7*B45</f>
-        <v>1191.4000000000001</v>
+        <v>2268.1</v>
       </c>
       <c r="C46" s="22">
         <f t="shared" si="1"/>
-        <v>1079.4000000000001</v>
+        <v>0</v>
       </c>
       <c r="D46" s="22">
         <f t="shared" si="1"/>
@@ -2978,15 +3051,15 @@
       </c>
       <c r="B49" s="23">
         <f>B123+B124</f>
-        <v>200.31953518182419</v>
+        <v>227.35227522366205</v>
       </c>
       <c r="C49" s="23">
         <f>C123+C124</f>
-        <v>150.41293818150814</v>
+        <v>149.71979100094819</v>
       </c>
       <c r="D49" s="23">
         <f>D123+D124</f>
-        <v>50.599744180876009</v>
+        <v>47.827155458636227</v>
       </c>
       <c r="E49" s="23">
         <f>E123+E124</f>
@@ -3008,15 +3081,15 @@
       </c>
       <c r="B50" s="23">
         <f>B125+B126</f>
-        <v>39.732626554474187</v>
+        <v>39.863976474484978</v>
       </c>
       <c r="C50" s="23">
         <f>C125+C126</f>
-        <v>29.800624884152146</v>
+        <v>29.795964711727471</v>
       </c>
       <c r="D50" s="23">
         <f>D125+D126</f>
-        <v>9.9365427815346692</v>
+        <v>9.9162676982393521</v>
       </c>
       <c r="E50" s="23">
         <f>E125+E126</f>
@@ -3024,7 +3097,7 @@
       </c>
       <c r="F50" s="23">
         <f>SUM(B50:E50)</f>
-        <v>116.25706871314375</v>
+        <v>116.36348337743455</v>
       </c>
       <c r="G50" s="2"/>
       <c r="H50" s="2" t="s">
@@ -3041,15 +3114,15 @@
       </c>
       <c r="B51" s="24">
         <f>IF(B19=0,0,B50/B19)</f>
-        <v>0.99331566386185466</v>
+        <v>0.99659941186212442</v>
       </c>
       <c r="C51" s="24">
         <f>IF(C19=0,0,C50/C19)</f>
-        <v>0.99335416280507149</v>
+        <v>0.99319882372424906</v>
       </c>
       <c r="D51" s="24">
         <f>IF(D19=0,0,D50/D19)</f>
-        <v>0.99365427815346696</v>
+        <v>0.99162676982393516</v>
       </c>
       <c r="E51" s="24">
         <f>IF(E19=0,0,E50/E19)</f>
@@ -3133,7 +3206,7 @@
       </c>
       <c r="B55" s="22">
         <f>SUMPRODUCT(PRICE,Q_TOTAL)</f>
-        <v>2899.6000000000004</v>
+        <v>2896.8999999999996</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
@@ -3175,7 +3248,7 @@
       </c>
       <c r="B57" s="22">
         <f>INTERCEPTOR_SPEND+SYSTEM_SPEND</f>
-        <v>7999.6</v>
+        <v>7996.9</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
@@ -3217,7 +3290,7 @@
       </c>
       <c r="B59" s="22">
         <f>BUDGET-TOTAL_SPEND</f>
-        <v>0.3999999999996362</v>
+        <v>3.1000000000003638</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" s="2"/>
@@ -3280,7 +3353,7 @@
       </c>
       <c r="B62" s="23">
         <f>PAC3_Q/16+MSE_Q/12</f>
-        <v>41.541666666666671</v>
+        <v>38.3125</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" s="2"/>
@@ -3301,7 +3374,7 @@
       </c>
       <c r="B63" s="23">
         <f>PATRIOT_LAUNCHERS*PATRIOT_BATTERIES-PATRIOT_LAUNCHERS_USED</f>
-        <v>6.4583333333333286</v>
+        <v>9.6875</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" s="2"/>
@@ -3343,7 +3416,7 @@
       </c>
       <c r="B65" s="26">
         <f>SUMPRODUCT(W,D)/SUMPRODUCT(W,RAID_SIZE)</f>
-        <v>0.97322318060097501</v>
+        <v>0.97511239623348023</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" s="2"/>
@@ -3376,11 +3449,11 @@
       </c>
       <c r="B67" s="21">
         <f t="shared" ref="B67:G67" si="2">B13*B160-B45</f>
-        <v>1678</v>
+        <v>1387</v>
       </c>
       <c r="C67" s="21">
         <f t="shared" si="2"/>
-        <v>1743</v>
+        <v>2000</v>
       </c>
       <c r="D67" s="21">
         <f t="shared" si="2"/>
@@ -3468,19 +3541,19 @@
       </c>
       <c r="B71" s="27">
         <f>IF(B9=0,0,B$17*IF(B$121=0,0,B$121*(1-EXP(-(B$123+B147)/B$121))-B$125)/B$7)</f>
-        <v>1.2414366916300577E-2</v>
+        <v>6.3156831138342475E-3</v>
       </c>
       <c r="C71" s="27">
         <f>IF(C9=0,0,B$17*IF(B$121=0,0,B$121*(1-EXP(-(B$123+C147)/B$121))-B$125)/C$7)</f>
-        <v>1.093646609293146E-2</v>
+        <v>5.5638160764730276E-3</v>
       </c>
       <c r="D71" s="27">
         <f>IF(D9=0,0,B$17*MAX(IF(B$121=0,0,B$121*(1-EXP(-(B$123+D147)/B$121))-B$125),IF(B$122=0,0,B$122*(1-EXP(-(B$124+D147)/B$122))-B$126))/D$7)</f>
-        <v>3.6167840622293021E-3</v>
+        <v>1.8400021670225764E-3</v>
       </c>
       <c r="E71" s="27">
         <f>IF(E9=0,0,B$17*MAX(IF(B$121=0,0,B$121*(1-EXP(-(B$123+E147)/B$121))-B$125),IF(B$122=0,0,B$122*(1-EXP(-(B$124+E147)/B$122))-B$126))/E$7)</f>
-        <v>1.6463497344197898E-3</v>
+        <v>8.3756371043680004E-4</v>
       </c>
       <c r="F71" s="27">
         <f>IF(F9=0,0,B$17*MAX(IF(B$121=0,0,B$121*(1-EXP(-(B$123+F147)/B$121))-B$125),IF(B$122=0,0,B$122*(1-EXP(-(B$124+F147)/B$122))-B$126))/F$7)</f>
@@ -3488,7 +3561,7 @@
       </c>
       <c r="G71" s="27">
         <f>IF(G9=0,0,B$17*MAX(IF(B$121=0,0,B$121*(1-EXP(-(B$123+G147)/B$121))-B$125),IF(B$122=0,0,B$122*(1-EXP(-(B$124+G147)/B$122))-B$126))/G$7)</f>
-        <v>7.0126958153148298E-3</v>
+        <v>3.5676377894941556E-3</v>
       </c>
       <c r="H71" s="2" t="s">
         <v>135</v>
@@ -3504,11 +3577,11 @@
       </c>
       <c r="B72" s="27">
         <f>IF(B10=0,0,C$17*IF(C$121=0,0,C$121*(1-EXP(-(C$123+B148)/C$121))-C$125)/B$7)</f>
-        <v>6.1536945126876332E-3</v>
+        <v>6.2975303036146872E-3</v>
       </c>
       <c r="C72" s="27">
         <f>IF(C10=0,0,C$17*IF(C$121=0,0,C$121*(1-EXP(-(C$123+C148)/C$121))-C$125)/C$7)</f>
-        <v>5.4211118326057718E-3</v>
+        <v>5.5478243150891291E-3</v>
       </c>
       <c r="D72" s="27">
         <f>IF(D10=0,0,C$17*MAX(IF(C$121=0,0,C$121*(1-EXP(-(C$123+D148)/C$121))-C$125),IF(C$122=0,0,C$122*(1-EXP(-(C$124+D148)/C$122))-C$126))/D$7)</f>
@@ -3520,11 +3593,11 @@
       </c>
       <c r="F72" s="27">
         <f>IF(F10=0,0,C$17*MAX(IF(C$121=0,0,C$121*(1-EXP(-(C$123+F148)/C$121))-C$125),IF(C$122=0,0,C$122*(1-EXP(-(C$124+F148)/C$122))-C$126))/F$7)</f>
-        <v>1.1106668144850852E-2</v>
+        <v>1.1366274206524071E-2</v>
       </c>
       <c r="G72" s="27">
         <f>IF(G10=0,0,C$17*MAX(IF(C$121=0,0,C$121*(1-EXP(-(C$123+G148)/C$121))-C$125),IF(C$122=0,0,C$122*(1-EXP(-(C$124+G148)/C$122))-C$126))/G$7)</f>
-        <v>3.4761327781594265E-3</v>
+        <v>3.5573835302861595E-3</v>
       </c>
       <c r="H72" s="2" t="s">
         <v>135</v>
@@ -3540,11 +3613,11 @@
       </c>
       <c r="B73" s="27">
         <f>IF(B11=0,0,D$17*IF(D$121=0,0,D$121*(1-EXP(-(D$123+B149)/D$121))-D$125)/B$7)</f>
-        <v>4.5940973902900539E-3</v>
+        <v>6.0619478493491264E-3</v>
       </c>
       <c r="C73" s="27">
         <f>IF(C11=0,0,D$17*IF(D$121=0,0,D$121*(1-EXP(-(D$123+C149)/D$121))-D$125)/C$7)</f>
-        <v>4.0471810343031423E-3</v>
+        <v>5.3402873910932784E-3</v>
       </c>
       <c r="D73" s="27">
         <f>IF(D11=0,0,D$17*MAX(IF(D$121=0,0,D$121*(1-EXP(-(D$123+D149)/D$121))-D$125),IF(D$122=0,0,D$122*(1-EXP(-(D$124+D149)/D$122))-D$126))/D$7)</f>
@@ -3556,11 +3629,11 @@
       </c>
       <c r="F73" s="27">
         <f>IF(F11=0,0,D$17*MAX(IF(D$121=0,0,D$121*(1-EXP(-(D$123+F149)/D$121))-D$125),IF(D$122=0,0,D$122*(1-EXP(-(D$124+F149)/D$122))-D$126))/F$7)</f>
-        <v>8.2917855336942445E-3</v>
+        <v>1.0941076606142328E-2</v>
       </c>
       <c r="G73" s="27">
         <f>IF(G11=0,0,D$17*MAX(IF(D$121=0,0,D$121*(1-EXP(-(D$123+G149)/D$121))-D$125),IF(D$122=0,0,D$122*(1-EXP(-(D$124+G149)/D$122))-D$126))/G$7)</f>
-        <v>2.5951389838279695E-3</v>
+        <v>3.424306418716301E-3</v>
       </c>
       <c r="H73" s="2" t="s">
         <v>135</v>
@@ -4172,10 +4245,10 @@
         <v>189</v>
       </c>
       <c r="B108" s="19">
-        <v>32</v>
+        <v>328</v>
       </c>
       <c r="C108" s="19">
-        <v>257</v>
+        <v>0</v>
       </c>
       <c r="D108" s="19">
         <v>0</v>
@@ -4201,7 +4274,7 @@
         <v>191</v>
       </c>
       <c r="B109" s="19">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C109" s="19">
         <v>0</v>
@@ -4230,7 +4303,7 @@
         <v>192</v>
       </c>
       <c r="B110" s="19">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C110" s="19">
         <v>0</v>
@@ -4381,7 +4454,7 @@
       </c>
       <c r="B118" s="21">
         <f>100000*PATRIOT_SITES_COVERED-SUM(QC)</f>
-        <v>1599325</v>
+        <v>1599291</v>
       </c>
       <c r="C118" s="2"/>
       <c r="D118" s="2"/>
@@ -4492,15 +4565,15 @@
       </c>
       <c r="B123" s="23">
         <f>SUMPRODUCT($B$147:$G$147,$B$108:$G$108)</f>
-        <v>200.31953518182419</v>
+        <v>227.35227522366205</v>
       </c>
       <c r="C123" s="23">
         <f>SUMPRODUCT($B$148:$G$148,$B$109:$G$109)</f>
-        <v>150.41293818150814</v>
+        <v>149.71979100094819</v>
       </c>
       <c r="D123" s="23">
         <f>SUMPRODUCT($B$149:$G$149,$B$110:$G$110)</f>
-        <v>50.599744180876009</v>
+        <v>47.827155458636227</v>
       </c>
       <c r="E123" s="23">
         <f>SUMPRODUCT($B$150:$G$150,$B$111:$G$111)</f>
@@ -4508,7 +4581,7 @@
       </c>
       <c r="F123" s="23">
         <f t="shared" si="3"/>
-        <v>467.87434687796315</v>
+        <v>491.44135101700124</v>
       </c>
       <c r="G123" s="2"/>
       <c r="H123" s="2" t="s">
@@ -4556,15 +4629,15 @@
       </c>
       <c r="B125" s="23">
         <f t="shared" ref="B125:E126" si="4">IF(B121=0,0,B121*(1-EXP(-B123/B121)))</f>
-        <v>39.732626554474187</v>
+        <v>39.863976474484978</v>
       </c>
       <c r="C125" s="23">
         <f t="shared" si="4"/>
-        <v>29.800624884152146</v>
+        <v>29.795964711727471</v>
       </c>
       <c r="D125" s="23">
         <f t="shared" si="4"/>
-        <v>9.9365427815346692</v>
+        <v>9.9162676982393521</v>
       </c>
       <c r="E125" s="23">
         <f t="shared" si="4"/>
@@ -4572,7 +4645,7 @@
       </c>
       <c r="F125" s="23">
         <f t="shared" si="3"/>
-        <v>116.25706871314375</v>
+        <v>116.36348337743455</v>
       </c>
       <c r="G125" s="2"/>
       <c r="H125" s="2" t="s">
@@ -5527,28 +5600,28 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="46" t="s">
         <v>275</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
     </row>
     <row r="3" spans="1:8" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="44" t="s">
+      <c r="A3" s="46" t="s">
         <v>276</v>
       </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="45"/>
-      <c r="H3" s="45"/>
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="35" t="s">
@@ -5590,7 +5663,7 @@
       </c>
       <c r="D6" s="37">
         <f>Scenarios!C13*100</f>
-        <v>91.564768170863132</v>
+        <v>91.602876170564841</v>
       </c>
       <c r="E6" t="b">
         <f t="shared" ref="E6:E14" si="0">ROUND(D6,0)=C6</f>
@@ -5602,7 +5675,7 @@
       </c>
       <c r="G6" s="37">
         <f t="shared" ref="G6:G14" si="1">D6/(F6/1000)</f>
-        <v>16.294982946124559</v>
+        <v>16.301764694363047</v>
       </c>
       <c r="H6" t="s">
         <v>285</v>
@@ -5622,11 +5695,11 @@
       </c>
       <c r="D7" s="37">
         <f>Scenarios!C14*100</f>
-        <v>88.496928853866237</v>
+        <v>88.578726426429583</v>
       </c>
       <c r="E7" t="b">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" s="38">
         <f>Scenarios!D14</f>
@@ -5634,7 +5707,7 @@
       </c>
       <c r="G7" s="37">
         <f t="shared" si="1"/>
-        <v>15.749026347854896</v>
+        <v>15.763583148211415</v>
       </c>
       <c r="H7" t="s">
         <v>286</v>
@@ -5654,7 +5727,7 @@
       </c>
       <c r="D8" s="37">
         <f>Scenarios!C15*100</f>
-        <v>49.000734304430935</v>
+        <v>49.13668977663518</v>
       </c>
       <c r="E8" t="b">
         <f t="shared" si="0"/>
@@ -5666,7 +5739,7 @@
       </c>
       <c r="G8" s="37">
         <f t="shared" si="1"/>
-        <v>8.7202331834479878</v>
+        <v>8.7444279927098485</v>
       </c>
       <c r="H8" t="s">
         <v>287</v>
@@ -5694,11 +5767,11 @@
       </c>
       <c r="F9" s="38">
         <f>Scenarios!D16</f>
-        <v>4120.5</v>
+        <v>3138.4</v>
       </c>
       <c r="G9" s="37">
         <f t="shared" si="1"/>
-        <v>16.382039905712197</v>
+        <v>21.508474200703258</v>
       </c>
       <c r="H9" t="s">
         <v>288</v>
@@ -5778,11 +5851,11 @@
         <v>A ballistic-heavy</v>
       </c>
       <c r="C12" s="36">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D12" s="37">
         <f>Scenarios!C19*100</f>
-        <v>97.322318060097501</v>
+        <v>97.511239623348018</v>
       </c>
       <c r="E12" t="b">
         <f t="shared" si="0"/>
@@ -5790,11 +5863,11 @@
       </c>
       <c r="F12" s="38">
         <f>Scenarios!D19</f>
-        <v>7999.6</v>
+        <v>7996.9</v>
       </c>
       <c r="G12" s="37">
         <f t="shared" si="1"/>
-        <v>12.165898052414809</v>
+        <v>12.193629984537512</v>
       </c>
       <c r="H12" t="s">
         <v>291</v>
@@ -5814,7 +5887,7 @@
       </c>
       <c r="D13" s="37">
         <f>Scenarios!C20*100</f>
-        <v>94.901427402312876</v>
+        <v>94.956451958619326</v>
       </c>
       <c r="E13" t="b">
         <f t="shared" si="0"/>
@@ -5826,7 +5899,7 @@
       </c>
       <c r="G13" s="37">
         <f t="shared" si="1"/>
-        <v>11.8629749996641</v>
+        <v>11.869853241158443</v>
       </c>
       <c r="H13" t="s">
         <v>292</v>
@@ -5846,7 +5919,7 @@
       </c>
       <c r="D14" s="37">
         <f>Scenarios!C21*100</f>
-        <v>58.955297540037236</v>
+        <v>59.258142564089475</v>
       </c>
       <c r="E14" t="b">
         <f t="shared" si="0"/>
@@ -5854,11 +5927,11 @@
       </c>
       <c r="F14" s="38">
         <f>Scenarios!D21</f>
-        <v>7616.6</v>
+        <v>7996.9</v>
       </c>
       <c r="G14" s="37">
         <f t="shared" si="1"/>
-        <v>7.7403693957982878</v>
+        <v>7.4101392494703546</v>
       </c>
       <c r="H14" t="s">
         <v>293</v>
@@ -5870,7 +5943,7 @@
       </c>
       <c r="E16" s="39" t="b">
         <f>AND(E6:E14)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -5931,7 +6004,7 @@
         <v>3.1</v>
       </c>
       <c r="C21" s="36">
-        <v>4.0999999999999996</v>
+        <v>3.1</v>
       </c>
       <c r="D21">
         <f>ROUND(MIN(F9:F11)/1000,1)</f>
@@ -5939,7 +6012,7 @@
       </c>
       <c r="E21">
         <f>ROUND(MAX(F9:F11)/1000,1)</f>
-        <v>4.0999999999999996</v>
+        <v>3.1</v>
       </c>
       <c r="F21" t="b">
         <f>AND(D21=B21,E21=C21)</f>
@@ -5952,14 +6025,14 @@
         <v>3 - optimal mix (up to 8 batteries)</v>
       </c>
       <c r="B22" s="36">
-        <v>7.6</v>
+        <v>8</v>
       </c>
       <c r="C22" s="36">
         <v>8</v>
       </c>
       <c r="D22">
         <f>ROUND(MIN(F12:F14)/1000,1)</f>
-        <v>7.6</v>
+        <v>8</v>
       </c>
       <c r="E22">
         <f>ROUND(MAX(F12:F14)/1000,1)</f>
@@ -5976,16 +6049,16 @@
       </c>
     </row>
     <row r="26" spans="1:8" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="44" t="s">
+      <c r="A26" s="46" t="s">
         <v>301</v>
       </c>
-      <c r="B26" s="45"/>
-      <c r="C26" s="45"/>
-      <c r="D26" s="45"/>
-      <c r="E26" s="45"/>
-      <c r="F26" s="45"/>
-      <c r="G26" s="45"/>
-      <c r="H26" s="45"/>
+      <c r="B26" s="47"/>
+      <c r="C26" s="47"/>
+      <c r="D26" s="47"/>
+      <c r="E26" s="47"/>
+      <c r="F26" s="47"/>
+      <c r="G26" s="47"/>
+      <c r="H26" s="47"/>
     </row>
     <row r="27" spans="1:8" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="35" t="s">
@@ -6069,14 +6142,14 @@
         <v>308</v>
       </c>
       <c r="C30" s="42">
-        <v>28.375</v>
+        <v>28.376999999999999</v>
       </c>
       <c r="D30" s="43">
         <v>1999.1</v>
       </c>
       <c r="E30" s="37">
         <f t="shared" si="2"/>
-        <v>14.193887249262168</v>
+        <v>14.194887699464759</v>
       </c>
       <c r="G30">
         <v>3</v>
@@ -6093,18 +6166,18 @@
         <v>71</v>
       </c>
       <c r="C31" s="42">
-        <v>70.349000000000004</v>
+        <v>70.350999999999999</v>
       </c>
       <c r="D31" s="43">
         <v>2997.7</v>
       </c>
       <c r="E31" s="37">
         <f t="shared" si="2"/>
-        <v>23.467658538212632</v>
+        <v>23.468325716382559</v>
       </c>
       <c r="F31" s="37">
         <f t="shared" ref="F31:F51" si="3">(C31-C28)/((D31-D28)/1000)</f>
-        <v>14.827827827827834</v>
+        <v>14.829829829829832</v>
       </c>
       <c r="G31">
         <v>4</v>
@@ -6149,18 +6222,18 @@
         <v>308</v>
       </c>
       <c r="C33" s="42">
-        <v>43.46</v>
+        <v>43.460999999999999</v>
       </c>
       <c r="D33" s="43">
-        <v>2999.6</v>
+        <v>2998.6</v>
       </c>
       <c r="E33" s="37">
         <f t="shared" si="2"/>
-        <v>14.488598479797306</v>
+        <v>14.493763756419664</v>
       </c>
       <c r="F33" s="37">
         <f t="shared" si="3"/>
-        <v>15.077461269365319</v>
+        <v>15.091545772886443</v>
       </c>
       <c r="G33">
         <v>1</v>
@@ -6188,7 +6261,7 @@
       </c>
       <c r="F34" s="37">
         <f t="shared" si="3"/>
-        <v>12.099270947767895</v>
+        <v>12.097273544392289</v>
       </c>
       <c r="G34">
         <v>7</v>
@@ -6208,15 +6281,15 @@
         <v>72.915999999999997</v>
       </c>
       <c r="D35" s="43">
-        <v>3999.9</v>
+        <v>3999.4</v>
       </c>
       <c r="E35" s="37">
         <f t="shared" si="2"/>
-        <v>18.229455736393408</v>
+        <v>18.231734760214032</v>
       </c>
       <c r="F35" s="37">
         <f t="shared" si="3"/>
-        <v>15.579884023195357</v>
+        <v>15.587676302890861</v>
       </c>
       <c r="G35">
         <v>7</v>
@@ -6233,18 +6306,18 @@
         <v>308</v>
       </c>
       <c r="C36" s="42">
-        <v>47.491999999999997</v>
+        <v>47.502000000000002</v>
       </c>
       <c r="D36" s="43">
         <v>3999.5</v>
       </c>
       <c r="E36" s="37">
         <f t="shared" si="2"/>
-        <v>11.874484310538817</v>
+        <v>11.876984623077886</v>
       </c>
       <c r="F36" s="37">
         <f t="shared" si="3"/>
-        <v>4.0324032403240286</v>
+        <v>4.0373663702667635</v>
       </c>
       <c r="G36">
         <v>3</v>
@@ -6261,18 +6334,18 @@
         <v>71</v>
       </c>
       <c r="C37" s="42">
-        <v>90.805999999999997</v>
+        <v>90.912000000000006</v>
       </c>
       <c r="D37" s="43">
         <v>4998.2</v>
       </c>
       <c r="E37" s="37">
         <f t="shared" si="2"/>
-        <v>18.167740386539155</v>
+        <v>18.188948021287665</v>
       </c>
       <c r="F37" s="37">
         <f t="shared" si="3"/>
-        <v>8.348678943154523</v>
+        <v>8.4547638110488474</v>
       </c>
       <c r="G37">
         <v>8</v>
@@ -6300,7 +6373,7 @@
       </c>
       <c r="F38" s="37">
         <f t="shared" si="3"/>
-        <v>13.723329660422724</v>
+        <v>13.71645975170205</v>
       </c>
       <c r="G38">
         <v>8</v>
@@ -6328,7 +6401,7 @@
       </c>
       <c r="F39" s="37">
         <f t="shared" si="3"/>
-        <v>3.8445378151260523</v>
+        <v>3.834533813525407</v>
       </c>
       <c r="G39">
         <v>5</v>
@@ -6345,18 +6418,18 @@
         <v>71</v>
       </c>
       <c r="C40" s="42">
-        <v>91.573999999999998</v>
+        <v>91.887</v>
       </c>
       <c r="D40" s="43">
-        <v>5378.8</v>
+        <v>5616.1</v>
       </c>
       <c r="E40" s="37">
         <f t="shared" si="2"/>
-        <v>17.024986985944821</v>
+        <v>16.361353964494935</v>
       </c>
       <c r="F40" s="37">
         <f t="shared" si="3"/>
-        <v>2.0178665265370466</v>
+        <v>1.5779252306198308</v>
       </c>
       <c r="G40">
         <v>8</v>
@@ -6373,18 +6446,18 @@
         <v>307</v>
       </c>
       <c r="C41" s="42">
-        <v>89.570999999999998</v>
+        <v>89.590999999999994</v>
       </c>
       <c r="D41" s="43">
         <v>5616.1</v>
       </c>
       <c r="E41" s="37">
         <f t="shared" si="2"/>
-        <v>15.94896814515411</v>
+        <v>15.952529335303856</v>
       </c>
       <c r="F41" s="37">
         <f t="shared" si="3"/>
-        <v>4.7823272374170509</v>
+        <v>4.8146949344553995</v>
       </c>
       <c r="G41">
         <v>8</v>
@@ -6401,18 +6474,18 @@
         <v>308</v>
       </c>
       <c r="C42" s="42">
-        <v>53.997999999999998</v>
+        <v>54.005000000000003</v>
       </c>
       <c r="D42" s="43">
         <v>5618</v>
       </c>
       <c r="E42" s="37">
         <f t="shared" si="2"/>
-        <v>9.6116055535777853</v>
+        <v>9.612851548593806</v>
       </c>
       <c r="F42" s="37">
         <f t="shared" si="3"/>
-        <v>4.3027952819518474</v>
+        <v>4.3141056713524044</v>
       </c>
       <c r="G42">
         <v>6</v>
@@ -6429,18 +6502,18 @@
         <v>71</v>
       </c>
       <c r="C43" s="42">
-        <v>91.686000000000007</v>
+        <v>92.064999999999998</v>
       </c>
       <c r="D43" s="43">
-        <v>5996.3</v>
+        <v>5997.2</v>
       </c>
       <c r="E43" s="37">
         <f t="shared" si="2"/>
-        <v>15.290429097943735</v>
+        <v>15.351330620956448</v>
       </c>
       <c r="F43" s="37">
         <f t="shared" si="3"/>
-        <v>0.18137651821863801</v>
+        <v>0.46706901075832469</v>
       </c>
       <c r="G43">
         <v>8</v>
@@ -6457,18 +6530,18 @@
         <v>307</v>
       </c>
       <c r="C44" s="42">
-        <v>90.347999999999999</v>
+        <v>90.382999999999996</v>
       </c>
       <c r="D44" s="43">
         <v>5997.2</v>
       </c>
       <c r="E44" s="37">
         <f t="shared" si="2"/>
-        <v>15.065030347495499</v>
+        <v>15.070866404322018</v>
       </c>
       <c r="F44" s="37">
         <f t="shared" si="3"/>
-        <v>2.0388349514563164</v>
+        <v>2.0781946995539302</v>
       </c>
       <c r="G44">
         <v>8</v>
@@ -6485,18 +6558,18 @@
         <v>308</v>
       </c>
       <c r="C45" s="42">
-        <v>55.103000000000002</v>
+        <v>55.115000000000002</v>
       </c>
       <c r="D45" s="43">
-        <v>5999.6</v>
+        <v>5997.6</v>
       </c>
       <c r="E45" s="37">
         <f t="shared" si="2"/>
-        <v>9.1844456297086481</v>
+        <v>9.1895091369881285</v>
       </c>
       <c r="F45" s="37">
         <f t="shared" si="3"/>
-        <v>2.8957023060796723</v>
+        <v>2.9241306638566869</v>
       </c>
       <c r="G45">
         <v>6</v>
@@ -6513,18 +6586,18 @@
         <v>71</v>
       </c>
       <c r="C46" s="42">
-        <v>95.212000000000003</v>
+        <v>95.257000000000005</v>
       </c>
       <c r="D46" s="43">
         <v>6999.9</v>
       </c>
       <c r="E46" s="37">
         <f t="shared" si="2"/>
-        <v>13.601908598694269</v>
+        <v>13.608337261960887</v>
       </c>
       <c r="F46" s="37">
         <f t="shared" si="3"/>
-        <v>3.5133519330410508</v>
+        <v>3.1834048070210508</v>
       </c>
       <c r="G46">
         <v>7</v>
@@ -6541,18 +6614,18 @@
         <v>307</v>
       </c>
       <c r="C47" s="42">
-        <v>91.424000000000007</v>
+        <v>91.504000000000005</v>
       </c>
       <c r="D47" s="43">
         <v>6999.3</v>
       </c>
       <c r="E47" s="37">
         <f t="shared" si="2"/>
-        <v>13.061877616333064</v>
+        <v>13.073307330733074</v>
       </c>
       <c r="F47" s="37">
         <f t="shared" si="3"/>
-        <v>1.0737451352160534</v>
+        <v>1.1186508332501834</v>
       </c>
       <c r="G47">
         <v>7</v>
@@ -6569,18 +6642,18 @@
         <v>308</v>
       </c>
       <c r="C48" s="42">
-        <v>58.83</v>
+        <v>58.866999999999997</v>
       </c>
       <c r="D48" s="43">
         <v>6997.9</v>
       </c>
       <c r="E48" s="37">
         <f t="shared" si="2"/>
-        <v>8.4068077566126984</v>
+        <v>8.4120950570885551</v>
       </c>
       <c r="F48" s="37">
         <f t="shared" si="3"/>
-        <v>3.7333466893719316</v>
+        <v>3.7508747375787244</v>
       </c>
       <c r="G48">
         <v>8</v>
@@ -6597,18 +6670,18 @@
         <v>71</v>
       </c>
       <c r="C49" s="42">
-        <v>97.322000000000003</v>
+        <v>97.510999999999996</v>
       </c>
       <c r="D49" s="43">
-        <v>7999.6</v>
+        <v>7996.9</v>
       </c>
       <c r="E49" s="37">
         <f t="shared" si="2"/>
-        <v>12.165858292914645</v>
+        <v>12.193600020007754</v>
       </c>
       <c r="F49" s="37">
         <f t="shared" si="3"/>
-        <v>2.1106331899569852</v>
+        <v>2.2607823470411139</v>
       </c>
       <c r="G49">
         <v>8</v>
@@ -6625,18 +6698,18 @@
         <v>307</v>
       </c>
       <c r="C50" s="42">
-        <v>94.900999999999996</v>
+        <v>94.956000000000003</v>
       </c>
       <c r="D50" s="43">
         <v>7999.8</v>
       </c>
       <c r="E50" s="37">
         <f t="shared" si="2"/>
-        <v>11.862921573039324</v>
+        <v>11.869796744918622</v>
       </c>
       <c r="F50" s="37">
         <f t="shared" si="3"/>
-        <v>3.4752623688155819</v>
+        <v>3.4502748625687141</v>
       </c>
       <c r="G50">
         <v>8</v>
@@ -6653,18 +6726,18 @@
         <v>308</v>
       </c>
       <c r="C51" s="42">
-        <v>58.954999999999998</v>
+        <v>59.258000000000003</v>
       </c>
       <c r="D51" s="43">
-        <v>7616.6</v>
+        <v>7996.9</v>
       </c>
       <c r="E51" s="37">
         <f t="shared" si="2"/>
-        <v>7.740330331118872</v>
+        <v>7.4101214220510458</v>
       </c>
       <c r="F51" s="37">
         <f t="shared" si="3"/>
-        <v>0.2020365282042991</v>
+        <v>0.39139139139139673</v>
       </c>
       <c r="G51">
         <v>8</v>
@@ -6685,7 +6758,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:N39"/>
   <sheetFormatPr defaultColWidth="8.68359375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -6693,7 +6766,7 @@
     <col min="3" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="11" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="8" width="11" customWidth="1"/>
+    <col min="7" max="8" width="60" customWidth="1"/>
     <col min="9" max="9" width="9" customWidth="1"/>
     <col min="10" max="10" width="10" customWidth="1"/>
     <col min="11" max="12" width="8" customWidth="1"/>
@@ -6852,7 +6925,7 @@
         <v>71</v>
       </c>
       <c r="C13" s="29">
-        <v>0.91564768170863131</v>
+        <v>0.9160287617056484</v>
       </c>
       <c r="D13" s="28">
         <v>5619.2</v>
@@ -6896,7 +6969,7 @@
         <v>307</v>
       </c>
       <c r="C14" s="29">
-        <v>0.8849692885386623</v>
+        <v>0.88578726426429588</v>
       </c>
       <c r="D14" s="28">
         <v>5619.2</v>
@@ -6940,7 +7013,7 @@
         <v>308</v>
       </c>
       <c r="C15" s="29">
-        <v>0.49000734304430932</v>
+        <v>0.49136689776635178</v>
       </c>
       <c r="D15" s="28">
         <v>5619.2</v>
@@ -6987,7 +7060,7 @@
         <v>0.67502195431487111</v>
       </c>
       <c r="D16" s="28">
-        <v>4120.5</v>
+        <v>3138.4</v>
       </c>
       <c r="E16" s="9">
         <v>1</v>
@@ -7005,13 +7078,13 @@
         <v>48</v>
       </c>
       <c r="J16" s="9">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="K16" s="9">
         <v>0</v>
       </c>
       <c r="L16" s="9">
-        <v>50</v>
+        <v>96</v>
       </c>
       <c r="M16" s="9">
         <v>0</v>
@@ -7116,10 +7189,10 @@
         <v>71</v>
       </c>
       <c r="C19" s="29">
-        <v>0.97322318060097501</v>
+        <v>0.97511239623348023</v>
       </c>
       <c r="D19" s="28">
-        <v>7999.6</v>
+        <v>7996.9</v>
       </c>
       <c r="E19" s="9">
         <v>1</v>
@@ -7128,10 +7201,10 @@
         <v>8</v>
       </c>
       <c r="G19" s="9">
-        <v>322</v>
+        <v>613</v>
       </c>
       <c r="H19" s="9">
-        <v>257</v>
+        <v>0</v>
       </c>
       <c r="I19" s="9">
         <v>0</v>
@@ -7160,7 +7233,7 @@
         <v>307</v>
       </c>
       <c r="C20" s="29">
-        <v>0.94901427402312877</v>
+        <v>0.94956451958619326</v>
       </c>
       <c r="D20" s="28">
         <v>7999.8</v>
@@ -7204,10 +7277,10 @@
         <v>308</v>
       </c>
       <c r="C21" s="29">
-        <v>0.58955297540037233</v>
+        <v>0.59258142564089478</v>
       </c>
       <c r="D21" s="28">
-        <v>7616.6</v>
+        <v>7996.9</v>
       </c>
       <c r="E21" s="9">
         <v>1</v>
@@ -7216,13 +7289,13 @@
         <v>8</v>
       </c>
       <c r="G21" s="9">
-        <v>98</v>
+        <v>613</v>
       </c>
       <c r="H21" s="9">
-        <v>218</v>
+        <v>0</v>
       </c>
       <c r="I21" s="9">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="J21" s="9">
         <v>0</v>
@@ -7286,6 +7359,270 @@
       </c>
       <c r="G27" s="6" t="s">
         <v>327</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A28" s="9">
+        <v>8000</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>328</v>
+      </c>
+      <c r="C28" s="9">
+        <v>0</v>
+      </c>
+      <c r="D28" s="44">
+        <v>0.91602300000000003</v>
+      </c>
+      <c r="E28" s="45">
+        <v>5619.2</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>329</v>
+      </c>
+      <c r="G28" s="9" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A29" s="9">
+        <v>8000</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>328</v>
+      </c>
+      <c r="C29" s="9">
+        <v>0</v>
+      </c>
+      <c r="D29" s="44">
+        <v>0.91602799999999995</v>
+      </c>
+      <c r="E29" s="45">
+        <v>5619.2</v>
+      </c>
+      <c r="F29" s="9" t="s">
+        <v>329</v>
+      </c>
+      <c r="G29" s="9" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A30" s="9">
+        <v>8000</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>328</v>
+      </c>
+      <c r="C30" s="9">
+        <v>0</v>
+      </c>
+      <c r="D30" s="44">
+        <v>0.62497100000000005</v>
+      </c>
+      <c r="E30" s="45">
+        <v>5619.2</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>332</v>
+      </c>
+      <c r="G30" s="9" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A31" s="9">
+        <v>8000</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>334</v>
+      </c>
+      <c r="C31" s="9">
+        <v>0</v>
+      </c>
+      <c r="D31" s="44">
+        <v>0.88578699999999999</v>
+      </c>
+      <c r="E31" s="45">
+        <v>5619.2</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>329</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A32" s="9">
+        <v>8000</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>336</v>
+      </c>
+      <c r="C32" s="9">
+        <v>0</v>
+      </c>
+      <c r="D32" s="44">
+        <v>0.491367</v>
+      </c>
+      <c r="E32" s="45">
+        <v>5619.2</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>329</v>
+      </c>
+      <c r="G32" s="9" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A33" s="9">
+        <v>8000</v>
+      </c>
+      <c r="B33" s="9" t="s">
+        <v>338</v>
+      </c>
+      <c r="C33" s="9">
+        <v>0</v>
+      </c>
+      <c r="D33" s="44">
+        <v>0.67502200000000001</v>
+      </c>
+      <c r="E33" s="45">
+        <v>4120.5</v>
+      </c>
+      <c r="F33" s="9" t="s">
+        <v>329</v>
+      </c>
+      <c r="G33" s="9" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A34" s="9">
+        <v>8000</v>
+      </c>
+      <c r="B34" s="9" t="s">
+        <v>338</v>
+      </c>
+      <c r="C34" s="9">
+        <v>0</v>
+      </c>
+      <c r="D34" s="44">
+        <v>0.67502200000000001</v>
+      </c>
+      <c r="E34" s="45">
+        <v>3138.4</v>
+      </c>
+      <c r="F34" s="9" t="s">
+        <v>329</v>
+      </c>
+      <c r="G34" s="9" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A35" s="9">
+        <v>8000</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>341</v>
+      </c>
+      <c r="C35" s="9">
+        <v>0</v>
+      </c>
+      <c r="D35" s="44">
+        <v>0.53314099999999998</v>
+      </c>
+      <c r="E35" s="45">
+        <v>3138.4</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>329</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A36" s="9">
+        <v>8000</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>343</v>
+      </c>
+      <c r="C36" s="9">
+        <v>0</v>
+      </c>
+      <c r="D36" s="44">
+        <v>0.42504500000000001</v>
+      </c>
+      <c r="E36" s="45">
+        <v>3138.4</v>
+      </c>
+      <c r="F36" s="9" t="s">
+        <v>329</v>
+      </c>
+      <c r="G36" s="9" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A37">
+        <v>8000</v>
+      </c>
+      <c r="B37" t="s">
+        <v>344</v>
+      </c>
+      <c r="C37">
+        <v>0</v>
+      </c>
+      <c r="F37" t="s">
+        <v>345</v>
+      </c>
+      <c r="G37" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A38">
+        <v>8000</v>
+      </c>
+      <c r="B38" t="s">
+        <v>347</v>
+      </c>
+      <c r="C38">
+        <v>0</v>
+      </c>
+      <c r="F38" t="s">
+        <v>345</v>
+      </c>
+      <c r="G38" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A39" s="9">
+        <v>8000</v>
+      </c>
+      <c r="B39" s="9" t="s">
+        <v>348</v>
+      </c>
+      <c r="C39" s="9">
+        <v>0</v>
+      </c>
+      <c r="D39" s="44">
+        <v>0.59191800000000006</v>
+      </c>
+      <c r="E39" s="45">
+        <v>7995.1</v>
+      </c>
+      <c r="F39" s="9" t="s">
+        <v>349</v>
+      </c>
+      <c r="G39" s="9" t="s">
+        <v>350</v>
       </c>
     </row>
   </sheetData>
@@ -7305,111 +7642,111 @@
   <sheetData>
     <row r="1" spans="1:2" ht="17.25" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
-        <v>328</v>
+        <v>351</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="7" t="s">
-        <v>329</v>
+        <v>352</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>330</v>
+        <v>353</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="7" t="s">
-        <v>331</v>
+        <v>354</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>332</v>
+        <v>355</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="7" t="s">
-        <v>333</v>
+        <v>356</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>334</v>
+        <v>357</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="7" t="s">
-        <v>335</v>
+        <v>358</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>336</v>
+        <v>359</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="7" t="s">
-        <v>337</v>
+        <v>360</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>338</v>
+        <v>361</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="7" t="s">
-        <v>339</v>
+        <v>362</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>340</v>
+        <v>363</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="7" t="s">
-        <v>341</v>
+        <v>364</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>342</v>
+        <v>365</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="7" t="s">
-        <v>343</v>
+        <v>366</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>344</v>
+        <v>367</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="7" t="s">
-        <v>345</v>
+        <v>368</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>346</v>
+        <v>369</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="7" t="s">
-        <v>347</v>
+        <v>370</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>348</v>
+        <v>371</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="7" t="s">
-        <v>349</v>
+        <v>372</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>350</v>
+        <v>373</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="7" t="s">
-        <v>351</v>
+        <v>374</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>352</v>
+        <v>375</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="7" t="s">
-        <v>353</v>
+        <v>376</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>354</v>
+        <v>377</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
@@ -7418,82 +7755,82 @@
     </row>
     <row r="17" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="7" t="s">
-        <v>355</v>
+        <v>378</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>356</v>
+        <v>379</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="7" t="s">
-        <v>357</v>
+        <v>380</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>358</v>
+        <v>381</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="7" t="s">
-        <v>359</v>
+        <v>382</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>360</v>
+        <v>383</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="7" t="s">
-        <v>361</v>
+        <v>384</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>362</v>
+        <v>385</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="7" t="s">
-        <v>363</v>
+        <v>386</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>364</v>
+        <v>387</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="7" t="s">
-        <v>365</v>
+        <v>388</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>366</v>
+        <v>389</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="7" t="s">
-        <v>367</v>
+        <v>390</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>368</v>
+        <v>391</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="7" t="s">
-        <v>369</v>
+        <v>392</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>370</v>
+        <v>393</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="7" t="s">
-        <v>371</v>
+        <v>394</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>372</v>
+        <v>395</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="7" t="s">
-        <v>373</v>
+        <v>396</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>374</v>
+        <v>397</v>
       </c>
     </row>
   </sheetData>

</xml_diff>